<commit_message>
Fase 155, PR 5: en el Centro de cargas se ven juntas las dos cargas de un modulo
- Modulo con dos archivos (Llamadas Unicas y de Salida, Tipificacion): selector
  arriba ("Unicas de ingreso" / "De salida", "Llamadas" / "WhatsApp"); cada
  opcion muestra su cuadricula de meses, Subir/Reemplazar y Descargar
  plantilla. Tokens de la pestana activa (AA en claro y oscuro).
- INSTRUCCIONES de esas 4 plantillas (y fichas regeneradas): que archivo va en
  cada carga y de que reporte de Wolkvox sale.
- v1.56.0 y CHANGELOG.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_LLAMADAS_SALIDA.xlsx
+++ b/server/plantillas/PLANTILLA_LLAMADAS_SALIDA.xlsx
@@ -433,7 +433,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -465,66 +465,57 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Cómo se sube</v>
+        <v>Archivos del módulo</v>
       </c>
       <c r="B4" t="str">
-        <v>Cargar Datos → cliente → este módulo. El sistema reconoce el archivo por sus columnas, no por el nombre de la hoja ni del archivo.</v>
+        <v>Este módulo lleva 2 archivos, cada uno en su propia carga del Centro de cargas: (1) "Únicas de ingreso" — contestadas: Wolkvox, CDR; no contestadas: Wolkvox, reporte por skill y servicio. (2) "De salida" — Wolkvox, CDR. Esta plantilla es la de "De salida".</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Cómo se sube</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Cargar Datos → cliente → este módulo. El sistema reconoce el archivo por sus columnas, no por el nombre de la hoja ni del archivo.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
         <v>Importante</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B6" t="str">
         <v>No cambie los nombres de las columnas. Los ejemplos de abajo son inventados: no los copie a la hoja de datos.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Columna</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Obligatoria</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Qué va</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Ejemplo (inventado)</v>
-      </c>
-      <c r="E7" t="str">
-        <v>También se acepta como</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>AGENT_NAME</v>
+        <v>Columna</v>
       </c>
       <c r="B8" t="str">
-        <v>Sí</v>
+        <v>Obligatoria</v>
       </c>
       <c r="C8" t="str">
-        <v>Asesor que hizo la llamada.</v>
+        <v>Qué va</v>
       </c>
       <c r="D8" t="str">
-        <v>Asesor Ejemplo Uno</v>
+        <v>Ejemplo (inventado)</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>También se acepta como</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>DATE</v>
+        <v>AGENT_NAME</v>
       </c>
       <c r="B9" t="str">
         <v>Sí</v>
       </c>
       <c r="C9" t="str">
-        <v>Fecha de la llamada.</v>
+        <v>Asesor que hizo la llamada.</v>
       </c>
       <c r="D9" t="str">
-        <v>2026-08-01</v>
+        <v>Asesor Ejemplo Uno</v>
       </c>
       <c r="E9" t="str">
         <v/>
@@ -532,16 +523,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>TELEPHONE</v>
+        <v>DATE</v>
       </c>
       <c r="B10" t="str">
         <v>Sí</v>
       </c>
       <c r="C10" t="str">
-        <v>Número llamado. Solo se usa en el navegador; nunca se envía ni se guarda.</v>
+        <v>Fecha de la llamada.</v>
       </c>
       <c r="D10" t="str">
-        <v>3000000001</v>
+        <v>2026-08-01</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -549,16 +540,16 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>DESCRIPTION_COD_ACT</v>
+        <v>TELEPHONE</v>
       </c>
       <c r="B11" t="str">
         <v>Sí</v>
       </c>
       <c r="C11" t="str">
-        <v>Tipificación de la llamada.</v>
+        <v>Número llamado. Solo se usa en el navegador; nunca se envía ni se guarda.</v>
       </c>
       <c r="D11" t="str">
-        <v>Seguimiento</v>
+        <v>3000000001</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -566,24 +557,41 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SKILL_ID</v>
+        <v>DESCRIPTION_COD_ACT</v>
       </c>
       <c r="B12" t="str">
         <v>Sí</v>
       </c>
       <c r="C12" t="str">
-        <v>"LLAMADAS DE SALIDA CONECTADAS" o "LLAMADAS DE SALIDA NO CONECTADAS".</v>
+        <v>Tipificación de la llamada.</v>
       </c>
       <c r="D12" t="str">
-        <v>LLAMADAS DE SALIDA CONECTADAS</v>
+        <v>Seguimiento</v>
       </c>
       <c r="E12" t="str">
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>SKILL_ID</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="C13" t="str">
+        <v>"LLAMADAS DE SALIDA CONECTADAS" o "LLAMADAS DE SALIDA NO CONECTADAS".</v>
+      </c>
+      <c r="D13" t="str">
+        <v>LLAMADAS DE SALIDA CONECTADAS</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fase 163 (4): Llamadas de Salida con la plantilla de Edwin (TIPO), DATE con hora, '-' = Sin tipificacion (v1.61.0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_LLAMADAS_SALIDA.xlsx
+++ b/server/plantillas/PLANTILLA_LLAMADAS_SALIDA.xlsx
@@ -421,7 +421,7 @@
         <v>DESCRIPTION_COD_ACT</v>
       </c>
       <c r="E1" t="str">
-        <v>SKILL_ID</v>
+        <v>TIPO</v>
       </c>
     </row>
   </sheetData>
@@ -452,7 +452,7 @@
         <v>De dónde sale</v>
       </c>
       <c r="B2" t="str">
-        <v>Wolkvox: CDR → "1. Detalle de las llamadas" (salientes conectadas) + "5. Detalle de las llamadas para las no conectadas", con SKILL_ID diciendo cuál es cuál.</v>
+        <v>Wolkvox, dos reportes en una sola hoja: las CONECTADAS salen del CDR → "1. Detalle de las llamadas" (solo las de salida) y las NO CONECTADAS del reporte "5. Detalle de llamadas no conectadas". La columna TIPO dice cuál es cuál: "Conectada" o "No conectada".</v>
       </c>
     </row>
     <row r="3">
@@ -529,10 +529,10 @@
         <v>Sí</v>
       </c>
       <c r="C10" t="str">
-        <v>Fecha de la llamada.</v>
+        <v>Fecha y hora de la llamada. Cuenta el día en hora de Colombia.</v>
       </c>
       <c r="D10" t="str">
-        <v>2026-08-01</v>
+        <v>2026-08-01 09:30</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -563,7 +563,7 @@
         <v>Sí</v>
       </c>
       <c r="C12" t="str">
-        <v>Tipificación de la llamada.</v>
+        <v>Tipificación de la llamada. "-" o vacío = "Sin tipificación".</v>
       </c>
       <c r="D12" t="str">
         <v>Seguimiento</v>
@@ -574,19 +574,19 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>SKILL_ID</v>
+        <v>TIPO</v>
       </c>
       <c r="B13" t="str">
         <v>Sí</v>
       </c>
       <c r="C13" t="str">
-        <v>"LLAMADAS DE SALIDA CONECTADAS" o "LLAMADAS DE SALIDA NO CONECTADAS".</v>
+        <v>"Conectada" (sale del CDR, numeral 1) o "No conectada" (sale del reporte "Detalle de llamadas no conectadas", numeral 5).</v>
       </c>
       <c r="D13" t="str">
-        <v>LLAMADAS DE SALIDA CONECTADAS</v>
+        <v>Conectada</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>SKILL_ID</v>
       </c>
     </row>
   </sheetData>

</xml_diff>